<commit_message>
split three recycling processes
</commit_message>
<xml_diff>
--- a/SubRes_Tmpl/SubRES_Transport_trans.xlsx
+++ b/SubRes_Tmpl/SubRES_Transport_trans.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook" updateLinks="never"/>
   <bookViews>
-    <workbookView windowWidth="18340" windowHeight="8720" activeTab="1"/>
+    <workbookView windowHeight="7070" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="TechSelection" sheetId="21" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="181">
   <si>
     <t>~TFM_AVA</t>
   </si>
@@ -439,9 +439,6 @@
   </si>
   <si>
     <t>Saudi Arabia</t>
-  </si>
-  <si>
-    <t>XXXX</t>
   </si>
   <si>
     <t>\I:</t>
@@ -11896,40 +11893,40 @@
         <v>134</v>
       </c>
       <c r="AO66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AP66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AQ66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AR66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AS66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AT66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AU66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AV66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AW66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AX66" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="AP66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AQ66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AR66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AS66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AT66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AU66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AV66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AW66" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AX66" s="11" t="s">
+      <c r="AY66" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AY66" s="2" t="s">
+      <c r="AZ66" s="16" t="s">
         <v>137</v>
-      </c>
-      <c r="AZ66" s="16" t="s">
-        <v>138</v>
       </c>
       <c r="BE66" s="11"/>
       <c r="BF66" s="11"/>
@@ -11945,7 +11942,7 @@
         <v>68</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D67" s="2">
         <f t="shared" ref="D67:AK67" si="2">D77/1000</f>
@@ -12083,19 +12080,17 @@
         <v>0</v>
       </c>
       <c r="AL67" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AN67" s="15"/>
+      <c r="AX67" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="AN67" s="15">
-        <v>1000</v>
-      </c>
-      <c r="AX67" s="1" t="s">
+      <c r="AY67" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="AY67" s="1" t="s">
+      <c r="AZ67" s="16" t="s">
         <v>142</v>
-      </c>
-      <c r="AZ67" s="16" t="s">
-        <v>143</v>
       </c>
       <c r="BD67" s="17"/>
       <c r="BE67" s="11"/>
@@ -12246,17 +12241,15 @@
         <v>0</v>
       </c>
       <c r="AL68" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AN68" s="15">
-        <v>0</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="AN68" s="15"/>
       <c r="AX68" s="1"/>
       <c r="AY68" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AZ68" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="69" s="2" customFormat="1" ht="16" spans="3:52">
@@ -12398,17 +12391,15 @@
         <v>0</v>
       </c>
       <c r="AL69" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AN69" s="15">
-        <v>0</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="AN69" s="15"/>
       <c r="AX69" s="1"/>
       <c r="AY69" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AZ69" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="70" s="2" customFormat="1" ht="16" spans="3:52">
@@ -12550,17 +12541,15 @@
         <v>140000</v>
       </c>
       <c r="AL70" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AN70" s="15">
-        <v>0</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="AN70" s="15"/>
       <c r="AX70" s="1"/>
       <c r="AY70" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AZ70" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" s="2" customFormat="1" ht="16" spans="3:52">
@@ -12702,15 +12691,15 @@
         <v>0</v>
       </c>
       <c r="AL71" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AN71" s="15"/>
       <c r="AX71" s="1"/>
       <c r="AY71" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AZ71" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="72" s="2" customFormat="1" ht="16" spans="3:52">
@@ -12852,15 +12841,15 @@
         <v>0</v>
       </c>
       <c r="AL72" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AN72" s="15"/>
       <c r="AX72" s="1"/>
       <c r="AY72" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AZ72" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="73" s="1" customFormat="1" ht="16" spans="2:52">
@@ -13003,7 +12992,7 @@
         <v>0</v>
       </c>
       <c r="AL73" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AM73" s="2"/>
       <c r="AN73" s="15"/>
@@ -13017,16 +13006,16 @@
       <c r="AV73" s="2"/>
       <c r="AW73" s="2"/>
       <c r="AY73" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AZ73" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="74" s="3" customFormat="1"/>
     <row r="75" s="3" customFormat="1" spans="5:5">
       <c r="E75" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="76" s="3" customFormat="1"/>
@@ -14023,7 +14012,7 @@
   <sheetData>
     <row r="1" spans="1:47">
       <c r="A1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B1" t="s">
         <v>56</v>
@@ -14035,25 +14024,25 @@
         <v>47</v>
       </c>
       <c r="E1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" t="s">
         <v>152</v>
-      </c>
-      <c r="F1" t="s">
-        <v>153</v>
       </c>
       <c r="G1" t="s">
         <v>79</v>
       </c>
       <c r="H1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" t="s">
         <v>154</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>155</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>156</v>
-      </c>
-      <c r="K1" t="s">
-        <v>157</v>
       </c>
       <c r="L1" t="s">
         <v>3</v>
@@ -14175,28 +14164,28 @@
         <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E2" t="s">
         <v>68</v>
       </c>
       <c r="F2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" t="s">
         <v>159</v>
       </c>
-      <c r="G2" t="s">
-        <v>160</v>
-      </c>
       <c r="H2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L2">
         <v>7</v>
@@ -14304,7 +14293,7 @@
         <v>4</v>
       </c>
       <c r="AU2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:47">
@@ -14315,31 +14304,31 @@
         <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E3" t="s">
         <v>68</v>
       </c>
       <c r="F3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" t="s">
         <v>159</v>
       </c>
-      <c r="G3" t="s">
-        <v>160</v>
-      </c>
       <c r="H3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L3">
         <v>15</v>
@@ -14447,7 +14436,7 @@
         <v>15</v>
       </c>
       <c r="AU3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:47">
@@ -14458,31 +14447,31 @@
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E4" t="s">
         <v>68</v>
       </c>
       <c r="F4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" t="s">
         <v>159</v>
       </c>
-      <c r="G4" t="s">
-        <v>160</v>
-      </c>
       <c r="H4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L4">
         <v>15</v>
@@ -14590,7 +14579,7 @@
         <v>15</v>
       </c>
       <c r="AU4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:47">
@@ -14604,28 +14593,28 @@
         <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E5" t="s">
         <v>68</v>
       </c>
       <c r="F5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" t="s">
         <v>159</v>
       </c>
-      <c r="G5" t="s">
-        <v>160</v>
-      </c>
       <c r="H5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L5">
         <v>15</v>
@@ -14733,7 +14722,7 @@
         <v>15</v>
       </c>
       <c r="AU5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:47">
@@ -14744,31 +14733,31 @@
         <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E6" t="s">
         <v>68</v>
       </c>
       <c r="F6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G6" t="s">
         <v>159</v>
       </c>
-      <c r="G6" t="s">
-        <v>160</v>
-      </c>
       <c r="H6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L6">
         <v>35</v>
@@ -14876,7 +14865,7 @@
         <v>20</v>
       </c>
       <c r="AU6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:47">
@@ -14890,28 +14879,28 @@
         <v>111</v>
       </c>
       <c r="D7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E7" t="s">
         <v>68</v>
       </c>
       <c r="F7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G7" t="s">
         <v>159</v>
       </c>
-      <c r="G7" t="s">
-        <v>160</v>
-      </c>
       <c r="H7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L7">
         <v>35</v>
@@ -15019,7 +15008,7 @@
         <v>20</v>
       </c>
       <c r="AU7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:47">
@@ -15030,31 +15019,31 @@
         <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E8" t="s">
         <v>68</v>
       </c>
       <c r="F8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" t="s">
         <v>159</v>
       </c>
-      <c r="G8" t="s">
-        <v>160</v>
-      </c>
       <c r="H8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L8">
         <v>35</v>
@@ -15162,7 +15151,7 @@
         <v>20</v>
       </c>
       <c r="AU8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:47">
@@ -15173,31 +15162,31 @@
         <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E9" t="s">
         <v>68</v>
       </c>
       <c r="F9" t="s">
+        <v>158</v>
+      </c>
+      <c r="G9" t="s">
         <v>159</v>
       </c>
-      <c r="G9" t="s">
-        <v>160</v>
-      </c>
       <c r="H9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L9">
         <v>35</v>
@@ -15305,7 +15294,7 @@
         <v>20</v>
       </c>
       <c r="AU9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:47">
@@ -15316,31 +15305,31 @@
         <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E10" t="s">
         <v>68</v>
       </c>
       <c r="F10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G10" t="s">
         <v>159</v>
       </c>
-      <c r="G10" t="s">
-        <v>160</v>
-      </c>
       <c r="H10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L10">
         <v>35</v>
@@ -15448,7 +15437,7 @@
         <v>20</v>
       </c>
       <c r="AU10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:47">
@@ -15459,31 +15448,31 @@
         <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E11" t="s">
         <v>68</v>
       </c>
       <c r="F11" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" t="s">
         <v>159</v>
       </c>
-      <c r="G11" t="s">
-        <v>160</v>
-      </c>
       <c r="H11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L11">
         <v>35</v>
@@ -15591,7 +15580,7 @@
         <v>20</v>
       </c>
       <c r="AU11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:47">
@@ -15602,31 +15591,31 @@
         <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E12" t="s">
         <v>68</v>
       </c>
       <c r="F12" t="s">
+        <v>158</v>
+      </c>
+      <c r="G12" t="s">
         <v>159</v>
       </c>
-      <c r="G12" t="s">
-        <v>160</v>
-      </c>
       <c r="H12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L12">
         <v>35</v>
@@ -15734,7 +15723,7 @@
         <v>20</v>
       </c>
       <c r="AU12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:47">
@@ -15745,31 +15734,31 @@
         <v>50</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E13" t="s">
         <v>68</v>
       </c>
       <c r="F13" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" t="s">
         <v>159</v>
       </c>
-      <c r="G13" t="s">
-        <v>160</v>
-      </c>
       <c r="H13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L13">
         <v>12</v>
@@ -15877,7 +15866,7 @@
         <v>12</v>
       </c>
       <c r="AU13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:47">
@@ -15888,31 +15877,31 @@
         <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
         <v>68</v>
       </c>
       <c r="F14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G14" t="s">
         <v>159</v>
       </c>
-      <c r="G14" t="s">
-        <v>160</v>
-      </c>
       <c r="H14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L14">
         <v>12</v>
@@ -16020,7 +16009,7 @@
         <v>12</v>
       </c>
       <c r="AU14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:47">
@@ -16031,31 +16020,31 @@
         <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E15" t="s">
         <v>68</v>
       </c>
       <c r="F15" t="s">
+        <v>158</v>
+      </c>
+      <c r="G15" t="s">
         <v>159</v>
       </c>
-      <c r="G15" t="s">
-        <v>160</v>
-      </c>
       <c r="H15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L15">
         <v>12</v>
@@ -16163,7 +16152,7 @@
         <v>12</v>
       </c>
       <c r="AU15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:47">
@@ -16174,31 +16163,31 @@
         <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E16" t="s">
         <v>68</v>
       </c>
       <c r="F16" t="s">
+        <v>158</v>
+      </c>
+      <c r="G16" t="s">
         <v>159</v>
       </c>
-      <c r="G16" t="s">
-        <v>160</v>
-      </c>
       <c r="H16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L16">
         <v>12</v>
@@ -16306,7 +16295,7 @@
         <v>12</v>
       </c>
       <c r="AU16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:47">
@@ -16320,28 +16309,28 @@
         <v>112</v>
       </c>
       <c r="D17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E17" t="s">
         <v>68</v>
       </c>
       <c r="F17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G17" t="s">
         <v>159</v>
       </c>
-      <c r="G17" t="s">
-        <v>160</v>
-      </c>
       <c r="H17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L17">
         <v>12</v>
@@ -16449,7 +16438,7 @@
         <v>12</v>
       </c>
       <c r="AU17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:47">
@@ -16460,31 +16449,31 @@
         <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E18" t="s">
         <v>68</v>
       </c>
       <c r="F18" t="s">
+        <v>158</v>
+      </c>
+      <c r="G18" t="s">
         <v>159</v>
       </c>
-      <c r="G18" t="s">
-        <v>160</v>
-      </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L18">
         <v>12</v>
@@ -16592,7 +16581,7 @@
         <v>12</v>
       </c>
       <c r="AU18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:47">
@@ -16603,31 +16592,31 @@
         <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E19" t="s">
         <v>68</v>
       </c>
       <c r="F19" t="s">
+        <v>158</v>
+      </c>
+      <c r="G19" t="s">
         <v>159</v>
       </c>
-      <c r="G19" t="s">
-        <v>160</v>
-      </c>
       <c r="H19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L19">
         <v>12</v>
@@ -16735,7 +16724,7 @@
         <v>12</v>
       </c>
       <c r="AU19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:47">
@@ -16746,31 +16735,31 @@
         <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E20" t="s">
         <v>68</v>
       </c>
       <c r="F20" t="s">
+        <v>158</v>
+      </c>
+      <c r="G20" t="s">
         <v>159</v>
       </c>
-      <c r="G20" t="s">
-        <v>160</v>
-      </c>
       <c r="H20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L20">
         <v>100</v>
@@ -16878,7 +16867,7 @@
         <v>35</v>
       </c>
       <c r="AU20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:47">
@@ -16892,28 +16881,28 @@
         <v>113</v>
       </c>
       <c r="D21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E21" t="s">
         <v>68</v>
       </c>
       <c r="F21" t="s">
+        <v>158</v>
+      </c>
+      <c r="G21" t="s">
         <v>159</v>
       </c>
-      <c r="G21" t="s">
-        <v>160</v>
-      </c>
       <c r="H21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L21">
         <v>100</v>
@@ -17021,7 +17010,7 @@
         <v>35</v>
       </c>
       <c r="AU21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22" spans="1:47">
@@ -17032,31 +17021,31 @@
         <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E22" t="s">
         <v>68</v>
       </c>
       <c r="F22" t="s">
+        <v>158</v>
+      </c>
+      <c r="G22" t="s">
         <v>159</v>
       </c>
-      <c r="G22" t="s">
-        <v>160</v>
-      </c>
       <c r="H22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L22">
         <v>100</v>
@@ -17164,7 +17153,7 @@
         <v>35</v>
       </c>
       <c r="AU22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" spans="1:47">
@@ -17175,31 +17164,31 @@
         <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E23" t="s">
         <v>68</v>
       </c>
       <c r="F23" t="s">
+        <v>158</v>
+      </c>
+      <c r="G23" t="s">
         <v>159</v>
       </c>
-      <c r="G23" t="s">
-        <v>160</v>
-      </c>
       <c r="H23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L23">
         <v>40</v>
@@ -17307,7 +17296,7 @@
         <v>15</v>
       </c>
       <c r="AU23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24" spans="1:47">
@@ -17321,28 +17310,28 @@
         <v>114</v>
       </c>
       <c r="D24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E24" t="s">
         <v>68</v>
       </c>
       <c r="F24" t="s">
+        <v>158</v>
+      </c>
+      <c r="G24" t="s">
         <v>159</v>
       </c>
-      <c r="G24" t="s">
-        <v>160</v>
-      </c>
       <c r="H24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L24">
         <v>40</v>
@@ -17450,7 +17439,7 @@
         <v>15</v>
       </c>
       <c r="AU24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:47">
@@ -17461,31 +17450,31 @@
         <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E25" t="s">
         <v>68</v>
       </c>
       <c r="F25" t="s">
+        <v>158</v>
+      </c>
+      <c r="G25" t="s">
         <v>159</v>
       </c>
-      <c r="G25" t="s">
-        <v>160</v>
-      </c>
       <c r="H25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L25">
         <v>40</v>
@@ -17593,7 +17582,7 @@
         <v>15</v>
       </c>
       <c r="AU25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:47">
@@ -17604,31 +17593,31 @@
         <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E26" t="s">
         <v>68</v>
       </c>
       <c r="F26" t="s">
+        <v>158</v>
+      </c>
+      <c r="G26" t="s">
         <v>159</v>
       </c>
-      <c r="G26" t="s">
-        <v>160</v>
-      </c>
       <c r="H26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L26">
         <v>40</v>
@@ -17736,7 +17725,7 @@
         <v>15</v>
       </c>
       <c r="AU26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="1:47">
@@ -17747,31 +17736,31 @@
         <v>50</v>
       </c>
       <c r="C27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E27" t="s">
         <v>68</v>
       </c>
       <c r="F27" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" t="s">
         <v>159</v>
       </c>
-      <c r="G27" t="s">
-        <v>160</v>
-      </c>
       <c r="H27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L27">
         <v>40</v>
@@ -17879,7 +17868,7 @@
         <v>15</v>
       </c>
       <c r="AU27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:47">
@@ -17890,31 +17879,31 @@
         <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E28" t="s">
         <v>68</v>
       </c>
       <c r="F28" t="s">
+        <v>158</v>
+      </c>
+      <c r="G28" t="s">
         <v>159</v>
       </c>
-      <c r="G28" t="s">
-        <v>160</v>
-      </c>
       <c r="H28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L28">
         <v>40</v>
@@ -18022,7 +18011,7 @@
         <v>15</v>
       </c>
       <c r="AU28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:47">
@@ -18036,28 +18025,28 @@
         <v>109</v>
       </c>
       <c r="D29" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" t="s">
+        <v>157</v>
+      </c>
+      <c r="F29" t="s">
         <v>158</v>
       </c>
-      <c r="E29" t="s">
-        <v>158</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>159</v>
       </c>
-      <c r="G29" t="s">
-        <v>160</v>
-      </c>
       <c r="H29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L29">
         <v>0.99</v>
@@ -18165,7 +18154,7 @@
         <v>0.99</v>
       </c>
       <c r="AU29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:47">
@@ -18176,31 +18165,31 @@
         <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D30" t="s">
+        <v>157</v>
+      </c>
+      <c r="E30" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" t="s">
         <v>158</v>
       </c>
-      <c r="E30" t="s">
-        <v>158</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>159</v>
       </c>
-      <c r="G30" t="s">
-        <v>160</v>
-      </c>
       <c r="H30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L30">
         <v>0.58697</v>
@@ -18308,7 +18297,7 @@
         <v>0.58697</v>
       </c>
       <c r="AU30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:47">
@@ -18319,31 +18308,31 @@
         <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D31" t="s">
+        <v>157</v>
+      </c>
+      <c r="E31" t="s">
+        <v>157</v>
+      </c>
+      <c r="F31" t="s">
         <v>158</v>
       </c>
-      <c r="E31" t="s">
-        <v>158</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>159</v>
       </c>
-      <c r="G31" t="s">
-        <v>160</v>
-      </c>
       <c r="H31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L31">
         <v>0.58697</v>
@@ -18451,7 +18440,7 @@
         <v>0.58697</v>
       </c>
       <c r="AU31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="32" spans="1:47">
@@ -18465,28 +18454,28 @@
         <v>110</v>
       </c>
       <c r="D32" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" t="s">
         <v>158</v>
       </c>
-      <c r="E32" t="s">
-        <v>158</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>159</v>
       </c>
-      <c r="G32" t="s">
-        <v>160</v>
-      </c>
       <c r="H32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L32">
         <v>0.58697</v>
@@ -18594,7 +18583,7 @@
         <v>0.58697</v>
       </c>
       <c r="AU32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:47">
@@ -18605,31 +18594,31 @@
         <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D33" t="s">
+        <v>157</v>
+      </c>
+      <c r="E33" t="s">
+        <v>157</v>
+      </c>
+      <c r="F33" t="s">
         <v>158</v>
       </c>
-      <c r="E33" t="s">
-        <v>158</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>159</v>
       </c>
-      <c r="G33" t="s">
-        <v>160</v>
-      </c>
       <c r="H33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L33">
         <v>0.07207</v>
@@ -18737,7 +18726,7 @@
         <v>0.07207</v>
       </c>
       <c r="AU33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:47">
@@ -18751,28 +18740,28 @@
         <v>111</v>
       </c>
       <c r="D34" t="s">
+        <v>157</v>
+      </c>
+      <c r="E34" t="s">
+        <v>157</v>
+      </c>
+      <c r="F34" t="s">
         <v>158</v>
       </c>
-      <c r="E34" t="s">
-        <v>158</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>159</v>
       </c>
-      <c r="G34" t="s">
-        <v>160</v>
-      </c>
       <c r="H34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L34">
         <v>0.07207</v>
@@ -18880,7 +18869,7 @@
         <v>0.07207</v>
       </c>
       <c r="AU34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="35" spans="1:47">
@@ -18891,31 +18880,31 @@
         <v>61</v>
       </c>
       <c r="C35" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D35" t="s">
+        <v>157</v>
+      </c>
+      <c r="E35" t="s">
+        <v>157</v>
+      </c>
+      <c r="F35" t="s">
         <v>158</v>
       </c>
-      <c r="E35" t="s">
-        <v>158</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>159</v>
       </c>
-      <c r="G35" t="s">
-        <v>160</v>
-      </c>
       <c r="H35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L35">
         <v>0.313</v>
@@ -19023,7 +19012,7 @@
         <v>0.313</v>
       </c>
       <c r="AU35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:47">
@@ -19034,31 +19023,31 @@
         <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D36" t="s">
+        <v>157</v>
+      </c>
+      <c r="E36" t="s">
+        <v>157</v>
+      </c>
+      <c r="F36" t="s">
         <v>158</v>
       </c>
-      <c r="E36" t="s">
-        <v>158</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>159</v>
       </c>
-      <c r="G36" t="s">
-        <v>160</v>
-      </c>
       <c r="H36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L36">
         <v>0.08</v>
@@ -19166,7 +19155,7 @@
         <v>0.08</v>
       </c>
       <c r="AU36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:47">
@@ -19177,31 +19166,31 @@
         <v>61</v>
       </c>
       <c r="C37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D37" t="s">
+        <v>157</v>
+      </c>
+      <c r="E37" t="s">
+        <v>157</v>
+      </c>
+      <c r="F37" t="s">
         <v>158</v>
       </c>
-      <c r="E37" t="s">
-        <v>158</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>159</v>
       </c>
-      <c r="G37" t="s">
-        <v>160</v>
-      </c>
       <c r="H37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L37">
         <v>0.08</v>
@@ -19309,7 +19298,7 @@
         <v>0.08</v>
       </c>
       <c r="AU37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:47">
@@ -19320,31 +19309,31 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D38" t="s">
+        <v>157</v>
+      </c>
+      <c r="E38" t="s">
+        <v>157</v>
+      </c>
+      <c r="F38" t="s">
         <v>158</v>
       </c>
-      <c r="E38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>159</v>
       </c>
-      <c r="G38" t="s">
-        <v>160</v>
-      </c>
       <c r="H38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L38">
         <v>0.076</v>
@@ -19452,7 +19441,7 @@
         <v>0.076</v>
       </c>
       <c r="AU38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="39" spans="1:47">
@@ -19463,31 +19452,31 @@
         <v>61</v>
       </c>
       <c r="C39" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D39" t="s">
+        <v>157</v>
+      </c>
+      <c r="E39" t="s">
+        <v>157</v>
+      </c>
+      <c r="F39" t="s">
         <v>158</v>
       </c>
-      <c r="E39" t="s">
-        <v>158</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>159</v>
       </c>
-      <c r="G39" t="s">
-        <v>160</v>
-      </c>
       <c r="H39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L39">
         <v>0.0612</v>
@@ -19595,7 +19584,7 @@
         <v>0.0612</v>
       </c>
       <c r="AU39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="40" spans="1:47">
@@ -19606,31 +19595,31 @@
         <v>61</v>
       </c>
       <c r="C40" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D40" t="s">
+        <v>157</v>
+      </c>
+      <c r="E40" t="s">
+        <v>157</v>
+      </c>
+      <c r="F40" t="s">
         <v>158</v>
       </c>
-      <c r="E40" t="s">
-        <v>158</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>159</v>
       </c>
-      <c r="G40" t="s">
-        <v>160</v>
-      </c>
       <c r="H40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L40">
         <v>0.527722806887128</v>
@@ -19738,7 +19727,7 @@
         <v>0.527722806887128</v>
       </c>
       <c r="AU40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:47">
@@ -19749,31 +19738,31 @@
         <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D41" t="s">
+        <v>157</v>
+      </c>
+      <c r="E41" t="s">
+        <v>157</v>
+      </c>
+      <c r="F41" t="s">
         <v>158</v>
       </c>
-      <c r="E41" t="s">
-        <v>158</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>159</v>
       </c>
-      <c r="G41" t="s">
-        <v>160</v>
-      </c>
       <c r="H41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L41">
         <v>0.527722806887128</v>
@@ -19881,7 +19870,7 @@
         <v>0.527722806887128</v>
       </c>
       <c r="AU41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:47">
@@ -19892,31 +19881,31 @@
         <v>61</v>
       </c>
       <c r="C42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D42" t="s">
+        <v>157</v>
+      </c>
+      <c r="E42" t="s">
+        <v>157</v>
+      </c>
+      <c r="F42" t="s">
         <v>158</v>
       </c>
-      <c r="E42" t="s">
-        <v>158</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>159</v>
       </c>
-      <c r="G42" t="s">
-        <v>160</v>
-      </c>
       <c r="H42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L42">
         <v>1.16513217002889</v>
@@ -20024,7 +20013,7 @@
         <v>1.16513217002889</v>
       </c>
       <c r="AU42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" spans="1:47">
@@ -20035,31 +20024,31 @@
         <v>61</v>
       </c>
       <c r="C43" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D43" t="s">
+        <v>157</v>
+      </c>
+      <c r="E43" t="s">
+        <v>157</v>
+      </c>
+      <c r="F43" t="s">
         <v>158</v>
       </c>
-      <c r="E43" t="s">
-        <v>158</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>159</v>
       </c>
-      <c r="G43" t="s">
-        <v>160</v>
-      </c>
       <c r="H43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L43">
         <v>0.466052868011556</v>
@@ -20167,7 +20156,7 @@
         <v>0.466052868011556</v>
       </c>
       <c r="AU43" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="44" spans="1:47">
@@ -20181,28 +20170,28 @@
         <v>112</v>
       </c>
       <c r="D44" t="s">
+        <v>157</v>
+      </c>
+      <c r="E44" t="s">
+        <v>157</v>
+      </c>
+      <c r="F44" t="s">
         <v>158</v>
       </c>
-      <c r="E44" t="s">
-        <v>158</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>159</v>
       </c>
-      <c r="G44" t="s">
-        <v>160</v>
-      </c>
       <c r="H44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L44">
         <v>0.466052868011556</v>
@@ -20310,7 +20299,7 @@
         <v>0.466052868011556</v>
       </c>
       <c r="AU44" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:47">
@@ -20321,31 +20310,31 @@
         <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D45" t="s">
+        <v>157</v>
+      </c>
+      <c r="E45" t="s">
+        <v>157</v>
+      </c>
+      <c r="F45" t="s">
         <v>158</v>
       </c>
-      <c r="E45" t="s">
-        <v>158</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>159</v>
       </c>
-      <c r="G45" t="s">
-        <v>160</v>
-      </c>
       <c r="H45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L45">
         <v>0.475531491178995</v>
@@ -20453,7 +20442,7 @@
         <v>0.475531491178995</v>
       </c>
       <c r="AU45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="46" spans="1:47">
@@ -20464,31 +20453,31 @@
         <v>61</v>
       </c>
       <c r="C46" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D46" t="s">
+        <v>157</v>
+      </c>
+      <c r="E46" t="s">
+        <v>157</v>
+      </c>
+      <c r="F46" t="s">
         <v>158</v>
       </c>
-      <c r="E46" t="s">
-        <v>158</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>159</v>
       </c>
-      <c r="G46" t="s">
-        <v>160</v>
-      </c>
       <c r="H46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L46">
         <v>0.429345439465179</v>
@@ -20596,7 +20585,7 @@
         <v>0.429345439465179</v>
       </c>
       <c r="AU46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:47">
@@ -20607,31 +20596,31 @@
         <v>61</v>
       </c>
       <c r="C47" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D47" t="s">
+        <v>157</v>
+      </c>
+      <c r="E47" t="s">
+        <v>157</v>
+      </c>
+      <c r="F47" t="s">
         <v>158</v>
       </c>
-      <c r="E47" t="s">
-        <v>158</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>159</v>
       </c>
-      <c r="G47" t="s">
-        <v>160</v>
-      </c>
       <c r="H47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L47">
         <v>0.139365903767697</v>
@@ -20739,7 +20728,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="48" spans="1:47">
@@ -20753,28 +20742,28 @@
         <v>113</v>
       </c>
       <c r="D48" t="s">
+        <v>157</v>
+      </c>
+      <c r="E48" t="s">
+        <v>157</v>
+      </c>
+      <c r="F48" t="s">
         <v>158</v>
       </c>
-      <c r="E48" t="s">
-        <v>158</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>159</v>
       </c>
-      <c r="G48" t="s">
-        <v>160</v>
-      </c>
       <c r="H48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L48">
         <v>0.139365903767697</v>
@@ -20882,7 +20871,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU48" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:47">
@@ -20893,31 +20882,31 @@
         <v>61</v>
       </c>
       <c r="C49" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D49" t="s">
+        <v>157</v>
+      </c>
+      <c r="E49" t="s">
+        <v>157</v>
+      </c>
+      <c r="F49" t="s">
         <v>158</v>
       </c>
-      <c r="E49" t="s">
-        <v>158</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>159</v>
       </c>
-      <c r="G49" t="s">
-        <v>160</v>
-      </c>
       <c r="H49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L49">
         <v>0.139365903767697</v>
@@ -21025,7 +21014,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="50" spans="1:47">
@@ -21036,31 +21025,31 @@
         <v>61</v>
       </c>
       <c r="C50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D50" t="s">
+        <v>157</v>
+      </c>
+      <c r="E50" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" t="s">
         <v>158</v>
       </c>
-      <c r="E50" t="s">
-        <v>158</v>
-      </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>159</v>
       </c>
-      <c r="G50" t="s">
-        <v>160</v>
-      </c>
       <c r="H50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L50">
         <v>0.379626024625345</v>
@@ -21168,7 +21157,7 @@
         <v>0.379626024625345</v>
       </c>
       <c r="AU50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="51" spans="1:47">
@@ -21182,28 +21171,28 @@
         <v>114</v>
       </c>
       <c r="D51" t="s">
+        <v>157</v>
+      </c>
+      <c r="E51" t="s">
+        <v>157</v>
+      </c>
+      <c r="F51" t="s">
         <v>158</v>
       </c>
-      <c r="E51" t="s">
-        <v>158</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>159</v>
       </c>
-      <c r="G51" t="s">
-        <v>160</v>
-      </c>
       <c r="H51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L51">
         <v>0.379626024625345</v>
@@ -21311,7 +21300,7 @@
         <v>0.379626024625345</v>
       </c>
       <c r="AU51" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="52" spans="1:47">
@@ -21322,31 +21311,31 @@
         <v>61</v>
       </c>
       <c r="C52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D52" t="s">
+        <v>157</v>
+      </c>
+      <c r="E52" t="s">
+        <v>157</v>
+      </c>
+      <c r="F52" t="s">
         <v>158</v>
       </c>
-      <c r="E52" t="s">
-        <v>158</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>159</v>
       </c>
-      <c r="G52" t="s">
-        <v>160</v>
-      </c>
       <c r="H52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L52">
         <v>0.745426473864409</v>
@@ -21454,7 +21443,7 @@
         <v>0.745426473864409</v>
       </c>
       <c r="AU52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="53" spans="1:47">
@@ -21465,31 +21454,31 @@
         <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D53" t="s">
+        <v>157</v>
+      </c>
+      <c r="E53" t="s">
+        <v>157</v>
+      </c>
+      <c r="F53" t="s">
         <v>158</v>
       </c>
-      <c r="E53" t="s">
-        <v>158</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
         <v>159</v>
       </c>
-      <c r="G53" t="s">
-        <v>160</v>
-      </c>
       <c r="H53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L53">
         <v>0.372713236932204</v>
@@ -21597,7 +21586,7 @@
         <v>0.372713236932204</v>
       </c>
       <c r="AU53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="54" spans="1:47">
@@ -21608,31 +21597,31 @@
         <v>61</v>
       </c>
       <c r="C54" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D54" t="s">
+        <v>157</v>
+      </c>
+      <c r="E54" t="s">
+        <v>157</v>
+      </c>
+      <c r="F54" t="s">
         <v>158</v>
       </c>
-      <c r="E54" t="s">
-        <v>158</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>159</v>
       </c>
-      <c r="G54" t="s">
-        <v>160</v>
-      </c>
       <c r="H54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L54">
         <v>0.440757335287194</v>
@@ -21740,7 +21729,7 @@
         <v>0.440757335287194</v>
       </c>
       <c r="AU54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:47">
@@ -21751,31 +21740,31 @@
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D55" t="s">
+        <v>157</v>
+      </c>
+      <c r="E55" t="s">
+        <v>157</v>
+      </c>
+      <c r="F55" t="s">
         <v>158</v>
       </c>
-      <c r="E55" t="s">
-        <v>158</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
         <v>159</v>
       </c>
-      <c r="G55" t="s">
-        <v>160</v>
-      </c>
       <c r="H55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L55">
         <v>0.329484430322726</v>
@@ -21883,7 +21872,7 @@
         <v>0.329484430322726</v>
       </c>
       <c r="AU55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revise alumium mining boundary for CN and NA
</commit_message>
<xml_diff>
--- a/SubRes_Tmpl/SubRES_Transport_trans.xlsx
+++ b/SubRes_Tmpl/SubRES_Transport_trans.xlsx
@@ -42,6 +42,50 @@
     <author>xli9</author>
   </authors>
   <commentList>
+    <comment ref="M71" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>xli9:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+https://www.lightmetalage.com/news/industry-news/smelting/decline-of-u-s-primary-aluminum-production-and-the-growth-of-secondary-aluminum/?utm_source=chatgpt.com</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA71" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>xli9:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+US750 ktonne, CAN 2.9 Mtonne: https://en.wikipedia.org/wiki/Aluminum_industry_in_the_United_States?utm_source=chatgpt.com; https://www.statista.com/statistics/312839/primary-aluminum-production-in-the-united-states/?utm_source=chatgpt.com</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="D101" authorId="0">
       <text>
         <r>
@@ -653,7 +697,7 @@
     <numFmt numFmtId="178" formatCode="0.0"/>
     <numFmt numFmtId="179" formatCode="0.000"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -845,6 +889,17 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -12625,7 +12680,9 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="M71" s="17"/>
+      <c r="M71" s="17">
+        <v>41500</v>
+      </c>
       <c r="N71" s="2">
         <f t="shared" ref="N71:AM71" si="11">L81/1000</f>
         <v>0</v>
@@ -12678,7 +12735,9 @@
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="AA71" s="17"/>
+      <c r="AA71" s="17">
+        <v>3650</v>
+      </c>
       <c r="AB71" s="2">
         <f t="shared" si="11"/>
         <v>0</v>

</xml_diff>

<commit_message>
EV stock calibrated upto 2024 - based on perplexity research; overall stock of cars was probably too high - Xiao to check
</commit_message>
<xml_diff>
--- a/SubRes_Tmpl/SubRES_Transport_trans.xlsx
+++ b/SubRes_Tmpl/SubRES_Transport_trans.xlsx
@@ -623,100 +623,100 @@
     <t>NCAP_COST</t>
   </si>
   <si>
+    <t>commodity_group</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>stage</t>
+  </si>
+  <si>
+    <t>sow</t>
+  </si>
+  <si>
+    <t>year2</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>ANNUAL</t>
+  </si>
+  <si>
+    <t>2019</t>
+  </si>
+  <si>
     <t>Trd_lcv_nga</t>
+  </si>
+  <si>
+    <t>Trd_lcv_gsl</t>
   </si>
   <si>
     <t>Trd_lcv_lpg</t>
   </si>
   <si>
-    <t>Trd_lcv_gsl</t>
+    <t>Trd_3w_bdl</t>
   </si>
   <si>
-    <t>Trd_lcv_elc</t>
+    <t>Trd_3w_dsl</t>
+  </si>
+  <si>
+    <t>Trd_bus_bdl</t>
+  </si>
+  <si>
+    <t>Trd_bus_elc</t>
+  </si>
+  <si>
+    <t>Trd_bus_eth</t>
+  </si>
+  <si>
+    <t>Trd_bus_gsl</t>
+  </si>
+  <si>
+    <t>Trd_bus_lpg</t>
+  </si>
+  <si>
+    <t>Trd_bus_nga</t>
+  </si>
+  <si>
+    <t>Trd_car_bdl</t>
+  </si>
+  <si>
+    <t>Trd_car_dsl</t>
+  </si>
+  <si>
+    <t>Trd_car_elc</t>
+  </si>
+  <si>
+    <t>Trd_car_eth</t>
+  </si>
+  <si>
+    <t>Trd_car_lpg</t>
+  </si>
+  <si>
+    <t>lim_type</t>
+  </si>
+  <si>
+    <t>time_slice</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>Trd_car_nga</t>
+  </si>
+  <si>
+    <t>Trd_hdt_bdl</t>
+  </si>
+  <si>
+    <t>Trd_hdt_gsl</t>
   </si>
   <si>
     <t>Trd_lcv_bdl</t>
   </si>
   <si>
-    <t>Trd_hdt_gsl</t>
-  </si>
-  <si>
-    <t>Trd_hdt_bdl</t>
-  </si>
-  <si>
-    <t>Trd_car_nga</t>
-  </si>
-  <si>
-    <t>scenario</t>
-  </si>
-  <si>
-    <t>time_slice</t>
-  </si>
-  <si>
-    <t>lim_type</t>
-  </si>
-  <si>
-    <t>Trd_car_lpg</t>
-  </si>
-  <si>
-    <t>Trd_car_eth</t>
-  </si>
-  <si>
-    <t>Trd_car_elc</t>
-  </si>
-  <si>
-    <t>Trd_car_dsl</t>
-  </si>
-  <si>
-    <t>Trd_car_bdl</t>
-  </si>
-  <si>
-    <t>Trd_bus_nga</t>
-  </si>
-  <si>
-    <t>Trd_bus_lpg</t>
-  </si>
-  <si>
-    <t>Trd_bus_gsl</t>
-  </si>
-  <si>
-    <t>Trd_bus_eth</t>
-  </si>
-  <si>
-    <t>Trd_bus_elc</t>
-  </si>
-  <si>
-    <t>Trd_bus_bdl</t>
-  </si>
-  <si>
-    <t>Trd_3w_dsl</t>
-  </si>
-  <si>
-    <t>Trd_3w_bdl</t>
-  </si>
-  <si>
-    <t>2019</t>
-  </si>
-  <si>
-    <t>ANNUAL</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>year2</t>
-  </si>
-  <si>
-    <t>sow</t>
-  </si>
-  <si>
-    <t>stage</t>
-  </si>
-  <si>
-    <t>currency</t>
-  </si>
-  <si>
-    <t>commodity_group</t>
+    <t>Trd_lcv_elc</t>
   </si>
 </sst>
 </file>
@@ -11265,7 +11265,7 @@
       </c>
       <c r="K36" t="str">
         <f>"*"&amp;ROUND(SUMIFS(RoadTra_BY!S$2:S$79,RoadTra_BY!$B$2:$B$79,'Road transport'!$C36,RoadTra_BY!$C$2:$C$79,'Road transport'!$BA36),3)</f>
-        <v>*0.699</v>
+        <v>*0.466</v>
       </c>
       <c r="L36" t="str">
         <f>"*"&amp;ROUND(SUMIFS(RoadTra_BY!T$2:T$79,RoadTra_BY!$B$2:$B$79,'Road transport'!$C36,RoadTra_BY!$C$2:$C$79,'Road transport'!$BA36),3)</f>
@@ -16147,7 +16147,7 @@
   <sheetData>
     <row r="1" spans="1:47" ht="12.5">
       <c r="A1" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="B1" t="s">
         <v>56</v>
@@ -16159,25 +16159,25 @@
         <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="F1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="G1" t="s">
         <v>79</v>
       </c>
       <c r="H1" t="s">
-        <v>190</v>
+        <v>159</v>
       </c>
       <c r="I1" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="J1" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="K1" t="s">
-        <v>187</v>
+        <v>162</v>
       </c>
       <c r="L1" t="s">
         <v>3</v>
@@ -16285,7 +16285,7 @@
         <v>38</v>
       </c>
       <c r="AU1" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:47" ht="12.5">
@@ -16299,28 +16299,28 @@
         <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E2" t="s">
         <v>68</v>
       </c>
       <c r="F2" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G2" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L2">
         <v>7</v>
@@ -16428,7 +16428,7 @@
         <v>4</v>
       </c>
       <c r="AU2" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:47" ht="12.5">
@@ -16439,31 +16439,31 @@
         <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="D3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E3" t="s">
         <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G3" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L3">
         <v>15</v>
@@ -16571,7 +16571,7 @@
         <v>15</v>
       </c>
       <c r="AU3" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:47" ht="12.5">
@@ -16582,31 +16582,31 @@
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E4" t="s">
         <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G4" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L4">
         <v>15</v>
@@ -16714,7 +16714,7 @@
         <v>15</v>
       </c>
       <c r="AU4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:47" ht="12.5">
@@ -16728,28 +16728,28 @@
         <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E5" t="s">
         <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G5" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L5">
         <v>15</v>
@@ -16857,7 +16857,7 @@
         <v>15</v>
       </c>
       <c r="AU5" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:47" ht="12.5">
@@ -16868,31 +16868,31 @@
         <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E6" t="s">
         <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G6" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L6">
         <v>35</v>
@@ -17000,7 +17000,7 @@
         <v>20</v>
       </c>
       <c r="AU6" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:47" ht="12.5">
@@ -17014,28 +17014,28 @@
         <v>111</v>
       </c>
       <c r="D7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E7" t="s">
         <v>68</v>
       </c>
       <c r="F7" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G7" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L7">
         <v>35</v>
@@ -17143,7 +17143,7 @@
         <v>20</v>
       </c>
       <c r="AU7" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:47" ht="12.5">
@@ -17154,31 +17154,31 @@
         <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E8" t="s">
         <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G8" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L8">
         <v>35</v>
@@ -17286,7 +17286,7 @@
         <v>20</v>
       </c>
       <c r="AU8" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:47" ht="12.5">
@@ -17297,31 +17297,31 @@
         <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E9" t="s">
         <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G9" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L9">
         <v>35</v>
@@ -17429,7 +17429,7 @@
         <v>20</v>
       </c>
       <c r="AU9" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:47" ht="12.5">
@@ -17440,31 +17440,31 @@
         <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E10" t="s">
         <v>68</v>
       </c>
       <c r="F10" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G10" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L10">
         <v>35</v>
@@ -17572,7 +17572,7 @@
         <v>20</v>
       </c>
       <c r="AU10" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:47" ht="12.5">
@@ -17586,28 +17586,28 @@
         <v>176</v>
       </c>
       <c r="D11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E11" t="s">
         <v>68</v>
       </c>
       <c r="F11" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G11" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L11">
         <v>35</v>
@@ -17715,7 +17715,7 @@
         <v>20</v>
       </c>
       <c r="AU11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:47" ht="12.5">
@@ -17726,31 +17726,31 @@
         <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E12" t="s">
         <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G12" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L12">
         <v>35</v>
@@ -17858,7 +17858,7 @@
         <v>20</v>
       </c>
       <c r="AU12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:47" ht="12.5">
@@ -17869,31 +17869,31 @@
         <v>50</v>
       </c>
       <c r="C13" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E13" t="s">
         <v>68</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G13" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L13">
         <v>12</v>
@@ -18001,7 +18001,7 @@
         <v>12</v>
       </c>
       <c r="AU13" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:47" ht="12.5">
@@ -18012,31 +18012,31 @@
         <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E14" t="s">
         <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G14" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L14">
         <v>12</v>
@@ -18144,7 +18144,7 @@
         <v>12</v>
       </c>
       <c r="AU14" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:47" ht="12.5">
@@ -18155,31 +18155,31 @@
         <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E15" t="s">
         <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G15" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L15">
         <v>12</v>
@@ -18287,7 +18287,7 @@
         <v>12</v>
       </c>
       <c r="AU15" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:47" ht="12.5">
@@ -18298,31 +18298,31 @@
         <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E16" t="s">
         <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G16" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L16">
         <v>12</v>
@@ -18430,7 +18430,7 @@
         <v>12</v>
       </c>
       <c r="AU16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:47" ht="12.5">
@@ -18444,28 +18444,28 @@
         <v>112</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E17" t="s">
         <v>68</v>
       </c>
       <c r="F17" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G17" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L17">
         <v>12</v>
@@ -18573,7 +18573,7 @@
         <v>12</v>
       </c>
       <c r="AU17" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:47" ht="12.5">
@@ -18584,31 +18584,31 @@
         <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="D18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E18" t="s">
         <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G18" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L18">
         <v>12</v>
@@ -18716,7 +18716,7 @@
         <v>12</v>
       </c>
       <c r="AU18" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:47" ht="12.5">
@@ -18727,31 +18727,31 @@
         <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="D19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E19" t="s">
         <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G19" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L19">
         <v>12</v>
@@ -18859,7 +18859,7 @@
         <v>12</v>
       </c>
       <c r="AU19" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:47" ht="12.5">
@@ -18870,31 +18870,31 @@
         <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="D20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E20" t="s">
         <v>68</v>
       </c>
       <c r="F20" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G20" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L20">
         <v>100</v>
@@ -19002,7 +19002,7 @@
         <v>35</v>
       </c>
       <c r="AU20" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:47" ht="12.5">
@@ -19016,28 +19016,28 @@
         <v>113</v>
       </c>
       <c r="D21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E21" t="s">
         <v>68</v>
       </c>
       <c r="F21" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G21" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L21">
         <v>100</v>
@@ -19145,7 +19145,7 @@
         <v>35</v>
       </c>
       <c r="AU21" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:47" ht="12.5">
@@ -19156,31 +19156,31 @@
         <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E22" t="s">
         <v>68</v>
       </c>
       <c r="F22" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G22" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L22">
         <v>100</v>
@@ -19288,7 +19288,7 @@
         <v>35</v>
       </c>
       <c r="AU22" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:47" ht="12.5">
@@ -19299,31 +19299,31 @@
         <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="D23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E23" t="s">
         <v>68</v>
       </c>
       <c r="F23" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G23" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L23">
         <v>40</v>
@@ -19431,7 +19431,7 @@
         <v>15</v>
       </c>
       <c r="AU23" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:47" ht="12.5">
@@ -19445,28 +19445,28 @@
         <v>114</v>
       </c>
       <c r="D24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E24" t="s">
         <v>68</v>
       </c>
       <c r="F24" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G24" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L24">
         <v>40</v>
@@ -19574,7 +19574,7 @@
         <v>15</v>
       </c>
       <c r="AU24" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="1:47" ht="12.5">
@@ -19585,31 +19585,31 @@
         <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>162</v>
+        <v>190</v>
       </c>
       <c r="D25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E25" t="s">
         <v>68</v>
       </c>
       <c r="F25" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G25" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L25">
         <v>40</v>
@@ -19717,7 +19717,7 @@
         <v>15</v>
       </c>
       <c r="AU25" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:47" ht="12.5">
@@ -19728,31 +19728,31 @@
         <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="D26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E26" t="s">
         <v>68</v>
       </c>
       <c r="F26" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G26" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L26">
         <v>40</v>
@@ -19860,7 +19860,7 @@
         <v>15</v>
       </c>
       <c r="AU26" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:47" ht="12.5">
@@ -19871,31 +19871,31 @@
         <v>50</v>
       </c>
       <c r="C27" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="D27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E27" t="s">
         <v>68</v>
       </c>
       <c r="F27" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G27" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L27">
         <v>40</v>
@@ -20003,7 +20003,7 @@
         <v>15</v>
       </c>
       <c r="AU27" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:47" ht="12.5">
@@ -20014,31 +20014,31 @@
         <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="D28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E28" t="s">
         <v>68</v>
       </c>
       <c r="F28" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G28" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L28">
         <v>40</v>
@@ -20146,7 +20146,7 @@
         <v>15</v>
       </c>
       <c r="AU28" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:47" ht="12.5">
@@ -20160,28 +20160,28 @@
         <v>109</v>
       </c>
       <c r="D29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F29" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G29" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L29">
         <v>0.98999999999999999</v>
@@ -20289,7 +20289,7 @@
         <v>0.98999999999999999</v>
       </c>
       <c r="AU29" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:47" ht="12.5">
@@ -20300,31 +20300,31 @@
         <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="D30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F30" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G30" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L30">
         <v>0.58696999999999999</v>
@@ -20432,7 +20432,7 @@
         <v>0.58696999999999999</v>
       </c>
       <c r="AU30" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:47" ht="12.5">
@@ -20443,31 +20443,31 @@
         <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F31" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G31" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L31">
         <v>0.58696999999999999</v>
@@ -20575,7 +20575,7 @@
         <v>0.58696999999999999</v>
       </c>
       <c r="AU31" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="32" spans="1:47" ht="12.5">
@@ -20589,28 +20589,28 @@
         <v>110</v>
       </c>
       <c r="D32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F32" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G32" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L32">
         <v>0.58696999999999999</v>
@@ -20718,7 +20718,7 @@
         <v>0.58696999999999999</v>
       </c>
       <c r="AU32" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="1:47" ht="12.5">
@@ -20729,31 +20729,31 @@
         <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F33" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G33" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L33">
         <v>0.072069999999999995</v>
@@ -20861,7 +20861,7 @@
         <v>0.072069999999999995</v>
       </c>
       <c r="AU33" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:47" ht="12.5">
@@ -20875,28 +20875,28 @@
         <v>111</v>
       </c>
       <c r="D34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F34" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G34" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L34">
         <v>0.072069999999999995</v>
@@ -21004,7 +21004,7 @@
         <v>0.072069999999999995</v>
       </c>
       <c r="AU34" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:47" ht="12.5">
@@ -21015,31 +21015,31 @@
         <v>61</v>
       </c>
       <c r="C35" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F35" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G35" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L35">
         <v>0.313</v>
@@ -21147,7 +21147,7 @@
         <v>0.313</v>
       </c>
       <c r="AU35" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:47" ht="12.5">
@@ -21158,31 +21158,31 @@
         <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F36" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G36" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L36">
         <v>0.080000000000000002</v>
@@ -21290,7 +21290,7 @@
         <v>0.080000000000000002</v>
       </c>
       <c r="AU36" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:47" ht="12.5">
@@ -21301,31 +21301,31 @@
         <v>61</v>
       </c>
       <c r="C37" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F37" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G37" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L37">
         <v>0.080000000000000002</v>
@@ -21433,7 +21433,7 @@
         <v>0.080000000000000002</v>
       </c>
       <c r="AU37" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:47" ht="12.5">
@@ -21447,28 +21447,28 @@
         <v>176</v>
       </c>
       <c r="D38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F38" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G38" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L38">
         <v>0.075999999999999998</v>
@@ -21576,7 +21576,7 @@
         <v>0.075999999999999998</v>
       </c>
       <c r="AU38" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="39" spans="1:47" ht="12.5">
@@ -21587,31 +21587,31 @@
         <v>61</v>
       </c>
       <c r="C39" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F39" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G39" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L39">
         <v>0.061199999999999997</v>
@@ -21719,7 +21719,7 @@
         <v>0.061199999999999997</v>
       </c>
       <c r="AU39" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="40" spans="1:47" ht="12.5">
@@ -21730,31 +21730,31 @@
         <v>61</v>
       </c>
       <c r="C40" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F40" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G40" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L40">
         <v>0.52772280688712803</v>
@@ -21778,7 +21778,7 @@
         <v>0.52772280688712803</v>
       </c>
       <c r="S40">
-        <v>0.79158421033069304</v>
+        <v>0.52772280688712803</v>
       </c>
       <c r="T40">
         <v>0.52772280688712803</v>
@@ -21862,7 +21862,7 @@
         <v>0.52772280688712803</v>
       </c>
       <c r="AU40" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="41" spans="1:47" ht="12.5">
@@ -21873,31 +21873,31 @@
         <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F41" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G41" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L41">
         <v>0.52772280688712803</v>
@@ -21921,7 +21921,7 @@
         <v>0.52772280688712803</v>
       </c>
       <c r="S41">
-        <v>0.79158421033069304</v>
+        <v>0.52772280688712803</v>
       </c>
       <c r="T41">
         <v>0.52772280688712803</v>
@@ -22005,7 +22005,7 @@
         <v>0.52772280688712803</v>
       </c>
       <c r="AU41" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="1:47" ht="12.5">
@@ -22016,139 +22016,139 @@
         <v>61</v>
       </c>
       <c r="C42" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F42" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G42" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="M42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="N42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="O42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="P42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="Q42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="R42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="S42">
-        <v>1.74769825504333</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="T42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="U42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="V42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="W42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="X42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="Y42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="Z42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AA42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AB42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AC42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AD42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AE42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AF42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AG42">
-        <v>0.69907930201733304</v>
+        <v>0.55926344161386699</v>
       </c>
       <c r="AH42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AI42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AJ42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AK42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AL42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AM42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AN42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AO42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AP42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AQ42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AR42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AS42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AT42">
-        <v>1.1651321700288899</v>
+        <v>0.93210573602311098</v>
       </c>
       <c r="AU42" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="43" spans="1:47" ht="12.5">
@@ -22159,31 +22159,31 @@
         <v>61</v>
       </c>
       <c r="C43" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F43" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G43" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L43">
         <v>0.46605286801155599</v>
@@ -22207,7 +22207,7 @@
         <v>0.46605286801155599</v>
       </c>
       <c r="S43">
-        <v>0.69907930201733304</v>
+        <v>0.46605286801155599</v>
       </c>
       <c r="T43">
         <v>0.46605286801155599</v>
@@ -22291,7 +22291,7 @@
         <v>0.46605286801155599</v>
       </c>
       <c r="AU43" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="44" spans="1:47" ht="12.5">
@@ -22305,28 +22305,28 @@
         <v>112</v>
       </c>
       <c r="D44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F44" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G44" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L44">
         <v>0.46605286801155599</v>
@@ -22350,7 +22350,7 @@
         <v>0.46605286801155599</v>
       </c>
       <c r="S44">
-        <v>0.69907930201733304</v>
+        <v>0.46605286801155599</v>
       </c>
       <c r="T44">
         <v>0.46605286801155599</v>
@@ -22434,7 +22434,7 @@
         <v>0.46605286801155599</v>
       </c>
       <c r="AU44" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="45" spans="1:47" ht="12.5">
@@ -22445,31 +22445,31 @@
         <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="D45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F45" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G45" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L45">
         <v>0.47553149117899501</v>
@@ -22493,7 +22493,7 @@
         <v>0.47553149117899501</v>
       </c>
       <c r="S45">
-        <v>0.71329723676849299</v>
+        <v>0.47553149117899501</v>
       </c>
       <c r="T45">
         <v>0.47553149117899501</v>
@@ -22577,7 +22577,7 @@
         <v>0.47553149117899501</v>
       </c>
       <c r="AU45" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:47" ht="12.5">
@@ -22588,31 +22588,31 @@
         <v>61</v>
       </c>
       <c r="C46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D46" t="s">
+        <v>164</v>
+      </c>
+      <c r="E46" t="s">
+        <v>164</v>
+      </c>
+      <c r="F46" t="s">
+        <v>165</v>
+      </c>
+      <c r="G46" t="s">
         <v>166</v>
       </c>
-      <c r="D46" t="s">
-        <v>185</v>
-      </c>
-      <c r="E46" t="s">
-        <v>185</v>
-      </c>
-      <c r="F46" t="s">
-        <v>184</v>
-      </c>
-      <c r="G46" t="s">
-        <v>183</v>
-      </c>
       <c r="H46" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I46" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J46" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K46" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L46">
         <v>0.429345439465179</v>
@@ -22636,7 +22636,7 @@
         <v>0.429345439465179</v>
       </c>
       <c r="S46">
-        <v>0.64401815919776795</v>
+        <v>0.429345439465179</v>
       </c>
       <c r="T46">
         <v>0.429345439465179</v>
@@ -22720,7 +22720,7 @@
         <v>0.429345439465179</v>
       </c>
       <c r="AU46" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" spans="1:47" ht="12.5">
@@ -22731,31 +22731,31 @@
         <v>61</v>
       </c>
       <c r="C47" t="s">
+        <v>187</v>
+      </c>
+      <c r="D47" t="s">
+        <v>164</v>
+      </c>
+      <c r="E47" t="s">
+        <v>164</v>
+      </c>
+      <c r="F47" t="s">
         <v>165</v>
       </c>
-      <c r="D47" t="s">
-        <v>185</v>
-      </c>
-      <c r="E47" t="s">
-        <v>185</v>
-      </c>
-      <c r="F47" t="s">
-        <v>184</v>
-      </c>
       <c r="G47" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H47" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I47" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J47" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K47" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L47">
         <v>0.139365903767697</v>
@@ -22863,7 +22863,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU47" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="48" spans="1:47" ht="12.5">
@@ -22877,28 +22877,28 @@
         <v>113</v>
       </c>
       <c r="D48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F48" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G48" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L48">
         <v>0.139365903767697</v>
@@ -23006,7 +23006,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU48" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:47" ht="12.5">
@@ -23017,31 +23017,31 @@
         <v>61</v>
       </c>
       <c r="C49" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F49" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G49" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L49">
         <v>0.139365903767697</v>
@@ -23149,7 +23149,7 @@
         <v>0.139365903767697</v>
       </c>
       <c r="AU49" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="50" spans="1:47" ht="12.5">
@@ -23160,31 +23160,31 @@
         <v>61</v>
       </c>
       <c r="C50" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="D50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F50" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G50" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L50">
         <v>0.379626024625345</v>
@@ -23292,7 +23292,7 @@
         <v>0.379626024625345</v>
       </c>
       <c r="AU50" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="51" spans="1:47" ht="12.5">
@@ -23306,28 +23306,28 @@
         <v>114</v>
       </c>
       <c r="D51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F51" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G51" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L51">
         <v>0.379626024625345</v>
@@ -23435,7 +23435,7 @@
         <v>0.379626024625345</v>
       </c>
       <c r="AU51" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="52" spans="1:47" ht="12.5">
@@ -23446,31 +23446,31 @@
         <v>61</v>
       </c>
       <c r="C52" t="s">
-        <v>162</v>
+        <v>190</v>
       </c>
       <c r="D52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F52" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G52" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L52">
         <v>0.74542647386440897</v>
@@ -23578,7 +23578,7 @@
         <v>0.74542647386440897</v>
       </c>
       <c r="AU52" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="53" spans="1:47" ht="12.5">
@@ -23589,31 +23589,31 @@
         <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="D53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F53" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G53" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L53">
         <v>0.37271323693220398</v>
@@ -23721,7 +23721,7 @@
         <v>0.37271323693220398</v>
       </c>
       <c r="AU53" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="54" spans="1:47" ht="12.5">
@@ -23732,31 +23732,31 @@
         <v>61</v>
       </c>
       <c r="C54" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="D54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F54" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G54" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L54">
         <v>0.44075733528719402</v>
@@ -23864,7 +23864,7 @@
         <v>0.44075733528719402</v>
       </c>
       <c r="AU54" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" spans="1:47" ht="12.5">
@@ -23875,31 +23875,31 @@
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F55" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="G55" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="H55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="I55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="J55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="K55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="L55">
         <v>0.32948443032272601</v>
@@ -24007,7 +24007,7 @@
         <v>0.32948443032272601</v>
       </c>
       <c r="AU55" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>